<commit_message>
Recalibration du modele et ajout de sklearn dans les requirements
</commit_message>
<xml_diff>
--- a/Outputs/Modelisation/comparaison_modèles.xlsx
+++ b/Outputs/Modelisation/comparaison_modèles.xlsx
@@ -462,222 +462,222 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2">
-        <v>0.5187529729192428</v>
+        <v>0.5791495426392816</v>
       </c>
       <c r="B2">
-        <v>0.3515364707682955</v>
+        <v>-24.51380274328266</v>
       </c>
       <c r="C2">
-        <v>2377.895751820425</v>
+        <v>152.4452436889148</v>
       </c>
       <c r="D2">
-        <v>2656.649757277189</v>
+        <v>286.4827648526326</v>
       </c>
       <c r="E2">
-        <v>5.234600242664553</v>
+        <v>0.598197321854894</v>
       </c>
       <c r="F2">
-        <v>5.281594134345903</v>
+        <v>1.654182461946295</v>
       </c>
       <c r="G2">
-        <v>12846520.07239272</v>
+        <v>121626.9827285142</v>
       </c>
       <c r="H2">
-        <v>12781206.54174983</v>
+        <v>194808.2193539513</v>
       </c>
       <c r="I2">
-        <v>19937902.42979349</v>
+        <v>161417.1863475312</v>
       </c>
       <c r="J2">
-        <v>16840209.81382717</v>
+        <v>193187.2176360064</v>
       </c>
       <c r="K2">
-        <v>47.60288705128818</v>
+        <v>44.90429384376617</v>
       </c>
       <c r="L2">
-        <v>45.62253666731279</v>
+        <v>49.20767306088407</v>
       </c>
       <c r="M2">
-        <v>23298.56759560067</v>
+        <v>1765.990141753887</v>
       </c>
       <c r="N2">
-        <v>21990.04754598521</v>
+        <v>1490.48992171129</v>
       </c>
     </row>
     <row r="3" spans="1:14">
       <c r="A3">
-        <v>0.9941284653659579</v>
+        <v>0.9220592999096687</v>
       </c>
       <c r="B3">
-        <v>0.8823225945313683</v>
+        <v>0.2282384827914946</v>
       </c>
       <c r="C3">
-        <v>304.555483181696</v>
+        <v>69.19076569973515</v>
       </c>
       <c r="D3">
-        <v>1216.422449924783</v>
+        <v>196.3556888691498</v>
       </c>
       <c r="E3">
-        <v>0.731678607668086</v>
+        <v>0.2759745119144907</v>
       </c>
       <c r="F3">
-        <v>1.353693447037917</v>
+        <v>0.8174641815495227</v>
       </c>
       <c r="G3">
-        <v>485841.4392722599</v>
+        <v>39610.54382373954</v>
       </c>
       <c r="H3">
-        <v>3224819.730986662</v>
+        <v>144973.4412642214</v>
       </c>
       <c r="I3">
-        <v>918276.5386928566</v>
+        <v>51800.3128812434</v>
       </c>
       <c r="J3">
-        <v>6486323.23165914</v>
+        <v>162499.3355381956</v>
       </c>
       <c r="K3">
-        <v>44.71424246769594</v>
+        <v>46.50801862390067</v>
       </c>
       <c r="L3">
-        <v>43.47095690379273</v>
+        <v>54.8790658882402</v>
       </c>
       <c r="M3">
-        <v>785.1159421881068</v>
+        <v>127.4425115041482</v>
       </c>
       <c r="N3">
-        <v>50.37503262578221</v>
+        <v>6.170846073139764</v>
       </c>
     </row>
     <row r="4" spans="1:14">
       <c r="A4">
-        <v>0.9153555698022705</v>
+        <v>0.8954080492723342</v>
       </c>
       <c r="B4">
-        <v>0.8486228902736481</v>
+        <v>-0.04757825186118203</v>
       </c>
       <c r="C4">
-        <v>1145.929548548493</v>
+        <v>81.90774180929537</v>
       </c>
       <c r="D4">
-        <v>1463.684295896648</v>
+        <v>222.5804237906225</v>
       </c>
       <c r="E4">
-        <v>4.476569766370375</v>
+        <v>0.3370198414610373</v>
       </c>
       <c r="F4">
-        <v>4.548332706119737</v>
+        <v>0.9883406356910622</v>
       </c>
       <c r="G4">
-        <v>4078455.850902852</v>
+        <v>55184.78904102876</v>
       </c>
       <c r="H4">
-        <v>5597540.202008037</v>
+        <v>167432.4948989066</v>
       </c>
       <c r="I4">
-        <v>6144268.617537266</v>
+        <v>66758.06855013814</v>
       </c>
       <c r="J4">
-        <v>8731413.921963189</v>
+        <v>151845.7517020919</v>
       </c>
       <c r="K4">
-        <v>50.31148925322244</v>
+        <v>48.86187273667873</v>
       </c>
       <c r="L4">
-        <v>48.95651612069523</v>
+        <v>56.13010842368641</v>
       </c>
       <c r="M4">
-        <v>1289.465592604498</v>
+        <v>124.892686616976</v>
       </c>
       <c r="N4">
-        <v>16.61758579722138</v>
+        <v>1.145284509932832</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5">
-        <v>0.8417840610227981</v>
+        <v>0.786790352631473</v>
       </c>
       <c r="B5">
-        <v>0.78544621585951</v>
+        <v>0.2072491053381403</v>
       </c>
       <c r="C5">
-        <v>1411.081149645971</v>
+        <v>108.4462157845446</v>
       </c>
       <c r="D5">
-        <v>1667.39792509774</v>
+        <v>195.7515265731513</v>
       </c>
       <c r="E5">
-        <v>4.654708986226136</v>
+        <v>0.4263928034971952</v>
       </c>
       <c r="F5">
-        <v>4.695275250326797</v>
+        <v>0.8079507772408051</v>
       </c>
       <c r="G5">
-        <v>5707336.889727776</v>
+        <v>82389.62604214411</v>
       </c>
       <c r="H5">
-        <v>6801885.628189373</v>
+        <v>147864.900525486</v>
       </c>
       <c r="I5">
-        <v>9168812.229751494</v>
+        <v>102082.4498456365</v>
       </c>
       <c r="J5">
-        <v>11034701.34049779</v>
+        <v>148012.7947341295</v>
       </c>
       <c r="K5">
-        <v>49.05278587702946</v>
+        <v>48.68080703569581</v>
       </c>
       <c r="L5">
-        <v>47.27014279253085</v>
+        <v>57.79816513761467</v>
       </c>
       <c r="M5">
-        <v>1506.556986813093</v>
+        <v>131.1234199746042</v>
       </c>
       <c r="N5">
-        <v>30.94915476506186</v>
+        <v>2.321206108153016</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6">
-        <v>0.7905056498287135</v>
+        <v>0.7020774742158256</v>
       </c>
       <c r="B6">
-        <v>0.720464908133826</v>
+        <v>0.273781012853435</v>
       </c>
       <c r="C6">
-        <v>1586.557253839199</v>
+        <v>126.2988687981358</v>
       </c>
       <c r="D6">
-        <v>1809.363604397372</v>
+        <v>183.0390302610194</v>
       </c>
       <c r="E6">
-        <v>4.56304597698646</v>
+        <v>0.4837511290939749</v>
       </c>
       <c r="F6">
-        <v>4.605559965926261</v>
+        <v>0.7359797086875927</v>
       </c>
       <c r="G6">
-        <v>6881612.916253977</v>
+        <v>99575.542775086</v>
       </c>
       <c r="H6">
-        <v>7924626.309363827</v>
+        <v>141681.4970128094</v>
       </c>
       <c r="I6">
-        <v>11956679.72985624</v>
+        <v>141189.5922139944</v>
       </c>
       <c r="J6">
-        <v>13712727.79247814</v>
+        <v>147964.3808122986</v>
       </c>
       <c r="K6">
-        <v>45.98887879801794</v>
+        <v>43.3781686497672</v>
       </c>
       <c r="L6">
-        <v>45.82283388253538</v>
+        <v>57.79816513761467</v>
       </c>
       <c r="M6">
-        <v>1677.778754631871</v>
+        <v>139.5521725295914</v>
       </c>
       <c r="N6">
-        <v>42.02276914266645</v>
+        <v>0.9186509119808653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>